<commit_message>
Author Ledger English markets: round 7 partial (CA)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/author-ledger/anglo/Author_Ledger_English_Markets_Leads.xlsx
+++ b/author-ledger/anglo/Author_Ledger_English_Markets_Leads.xlsx
@@ -8749,7 +8749,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Cliff Redford</t>
+          <t>Cordelia Strube</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -8759,17 +8759,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Far and Wild: Adventures of The Worldwide Vet</t>
+          <t>At Sea in a Sieve</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Memoir / animals nonfiction</t>
+          <t>Literary fiction</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -8795,22 +8795,22 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>https://ecwpress.com/products/far-and-wild</t>
+          <t>https://ecwpress.com/products/at-sea-in-a-sieve</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Far and Wild available from ECW September 29, 2026</t>
+          <t>New 560-page novel published by ECW Press, June 2026</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Ontario Veterinary College 1998 graduate who owns Wellington Veterinary Hospital in Markham, ON; known as The Worldwide Vet.</t>
+          <t>Divides her time between her Toronto home and a country house in Yarker, Ontario</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>High - vet adventure memoir, broad animal-lover appeal</t>
+          <t>Medium - established literary novelist (11 novels)</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -8835,14 +8835,14 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>Residence evidence: owns a vet hospital in Markham, ON per ECW page (practice location, not explicit 'lives in') - confirm.</t>
+          <t>Toronto/Yarker ON per ECW page; confirm she is not a major-prize winner (established author)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Cordelia Strube</t>
+          <t>Daniel Gawthrop</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -8852,22 +8852,22 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>At Sea in a Sieve</t>
+          <t>Cutting Edge</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Literary fiction</t>
+          <t>Nonfiction</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>publicity@ecwpress.com</t>
+          <t>cynara@arsenalpulp.com</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -8877,33 +8877,33 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://ecwpress.com/pages/media-press</t>
+          <t>https://arsenalpulp.com/Media-Review-Copies</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
-          <t>ECW Press</t>
+          <t>Arsenal Pulp Press</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>https://ecwpress.com/products/at-sea-in-a-sieve</t>
+          <t>https://arsenalpulp.com/Events</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>New 560-page novel published by ECW Press, June 2026</t>
+          <t>Fall 2026 launch at Another Story Bookshop Toronto (Oct 13) and Bowen Island Public Library talk (Oct 17, 2026)</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Divides her time between her Toronto home and a country house in Yarker, Ontario</t>
+          <t>Lives in New Westminster, BC; touring Cutting Edge in fall 2026</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>Medium - established literary novelist (11 novels)</t>
+          <t>Medium - nonfiction with active fall 2026 event tour</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -8928,14 +8928,14 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>Toronto/Yarker ON per ECW page; confirm she is not a major-prize winner (established author)</t>
+          <t>Date inferred from Oct 2026 launch events on arsenalpulp.com/Events - confirm exact pub month on arsenalpulp.com book page; cynara@ is Arsenal Pulp publicity contact</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Daniel Gawthrop</t>
+          <t>Dayle Furlong</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -8945,22 +8945,22 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Cutting Edge</t>
+          <t>Unto the Day</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Nonfiction</t>
+          <t>Historical fiction</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>cynara@arsenalpulp.com</t>
+          <t>publicity@dundurn.com</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -8970,33 +8970,33 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://arsenalpulp.com/Media-Review-Copies</t>
+          <t>https://www.dundurn.com/contact</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Arsenal Pulp Press</t>
+          <t>Dundurn Press</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>https://arsenalpulp.com/Events</t>
+          <t>https://www.dundurn.com/books_/t22117/a9781459757127-unto-the-day</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>Fall 2026 launch at Another Story Bookshop Toronto (Oct 13) and Bowen Island Public Library talk (Oct 17, 2026)</t>
+          <t>Historical novel about George Brown's household, Dundurn, September 2026</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>Lives in New Westminster, BC; touring Cutting Edge in fall 2026</t>
+          <t>Originally from Newfoundland, now lives in Toronto; previous books include the novel Saltwater Cowboys and poetry collection Open Slowly</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>Medium - nonfiction with active fall 2026 event tour</t>
+          <t>Medium - historical fiction with Canadian-history hook</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -9021,14 +9021,14 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>Date inferred from Oct 2026 launch events on arsenalpulp.com/Events - confirm exact pub month on arsenalpulp.com book page; cynara@ is Arsenal Pulp publicity contact</t>
+          <t>Lives in Toronto per Dundurn product page; publicity inbox is shared</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Dayle Furlong</t>
+          <t>Debbie Mason</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -9038,22 +9038,22 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Unto the Day</t>
+          <t>The Christmas Getaway</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Historical fiction</t>
+          <t>Holiday romantic comedy</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>publicity@dundurn.com</t>
+          <t>readforever@hbgusa.com</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -9063,33 +9063,33 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.dundurn.com/contact</t>
+          <t>https://www.hachettebookgroup.com/press-publicity/</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Dundurn Press</t>
+          <t>Forever (Hachette Book Group)</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>https://www.dundurn.com/books_/t22117/a9781459757127-unto-the-day</t>
+          <t>https://www.hachettebookgroup.com/titles/debbie-mason/the-christmas-getaway/9781538778081/</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>Historical novel about George Brown's household, Dundurn, September 2026</t>
+          <t>The Christmas Getaway (Oct 2026); her book inspired the Hallmark movie Welcome to Christmas</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>Originally from Newfoundland, now lives in Toronto; previous books include the novel Saltwater Cowboys and poetry collection Open Slowly</t>
+          <t>One of her books inspired the Hallmark movie Welcome to Christmas</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>Medium - historical fiction with Canadian-history hook</t>
+          <t>High - holiday romance, Hallmark tie-in</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -9114,14 +9114,14 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>Lives in Toronto per Dundurn product page; publicity inbox is shared</t>
+          <t>HBG contributor page mentions Ottawa, Canada; confirm residence; USA Today bestseller; readforever@hbgusa.com is Forever imprint publicity inbox (HBG press page) - Publisher type, not author's own | UP6: Residence: 'lives in Ottawa, Canada' stated on her pen-name page kensingtonbooks.com/?p=60205 (Debbie Mazzuca, older page) plus HBG/Hachette AU bios 'with her family in Ottawa, Canada'</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Debbie Mason</t>
+          <t>Dietrich Kalteis</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -9131,22 +9131,22 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>The Christmas Getaway</t>
+          <t>Rust and Bone: A Novel</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Holiday romantic comedy</t>
+          <t>Historical fiction</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>readforever@hbgusa.com</t>
+          <t>publicity@ecwpress.com</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -9156,33 +9156,33 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.hachettebookgroup.com/press-publicity/</t>
+          <t>https://ecwpress.com/pages/media-press</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Forever (Hachette Book Group)</t>
+          <t>ECW Press</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>https://www.hachettebookgroup.com/titles/debbie-mason/the-christmas-getaway/9781538778081/</t>
+          <t>https://ecwpress.com/products/rust-and-bone</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>The Christmas Getaway (Oct 2026); her book inspired the Hallmark movie Welcome to Christmas</t>
+          <t>Rust and Bone published by ECW Press March 2026</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>One of her books inspired the Hallmark movie Welcome to Christmas</t>
+          <t>Novel follows a German teenager who escapes Russian captivity at the end of WWII and meets a young woman in war-torn Germany.</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>High - holiday romance, Hallmark tie-in</t>
+          <t>Medium - established crime/historical mid-list novelist</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>HBG contributor page mentions Ottawa, Canada; confirm residence; USA Today bestseller; readforever@hbgusa.com is Forever imprint publicity inbox (HBG press page) - Publisher type, not author's own | UP6: Residence: 'lives in Ottawa, Canada' stated on her pen-name page kensingtonbooks.com/?p=60205 (Debbie Mazzuca, older page) plus HBG/Hachette AU bios 'with her family in Ottawa, Canada'</t>
+          <t>UPGRADE of ca6.jsonl NEEDS_REVIEW row (adds title/date): ECW author page says he lives in West Vancouver, BC; replace ca6 row.</t>
         </is>
       </c>
     </row>
@@ -47106,7 +47106,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Curtis Garner</t>
+          <t>Cliff Redford</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -47116,22 +47116,22 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Isaac</t>
+          <t>Far and Wild: Adventures of The Worldwide Vet</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Literary fiction (debut novel)</t>
+          <t>Memoir / animals nonfiction</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>cynara@arsenalpulp.com</t>
+          <t>publicity@ecwpress.com</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -47141,33 +47141,33 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://arsenalpulp.com/Media-Review-Copies</t>
+          <t>https://ecwpress.com/pages/media-press</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Arsenal Pulp Press</t>
+          <t>ECW Press</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>https://arsenalpulp.com/Books/I/Isaac</t>
+          <t>https://ecwpress.com/products/far-and-wild</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Debut novel, 2025 paperback, set in London</t>
+          <t>Far and Wild available from ECW September 29, 2026</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Debut novel set in London</t>
+          <t>Ontario Veterinary College 1998 graduate who owns Wellington Veterinary Hospital in Markham, ON; known as The Worldwide Vet.</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>Medium - LGBTQ+ literary debut</t>
+          <t>High - vet adventure memoir, broad animal-lover appeal</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -47192,14 +47192,14 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>Confirm residence; listed on arsenalpulp.com/Events per assignment but snippet gave no location | Review: Residence/nationality not stated in results (novel set in London - may not be Canadian)</t>
+          <t>Residence evidence: owns a vet hospital in Markham, ON per ECW page (practice location, not explicit 'lives in') - confirm. | Only workplace (vet hospital in Markham, ON) stated, not residence. | Review: Only workplace (vet hospital in Markham, ON) stated, not residence.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Denise Da Costa</t>
+          <t>Curtis Garner</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -47209,18 +47209,22 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>And the Walls Came Down</t>
+          <t>Isaac</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Fiction (debut novel)</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>Literary fiction (debut novel)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>publicity@dundurn.com</t>
+          <t>cynara@arsenalpulp.com</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -47230,33 +47234,33 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.dundurn.com/contact</t>
+          <t>https://arsenalpulp.com/Media-Review-Copies</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Dundurn Press</t>
+          <t>Arsenal Pulp Press</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>https://www.dundurn.com/blog_/t43181/p159409-essential-toronto-reading-list</t>
+          <t>https://arsenalpulp.com/Books/I/Isaac</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Dundurn title</t>
+          <t>Debut novel, 2025 paperback, set in London</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Debut novel about a woman returning to her hometown</t>
+          <t>Debut novel set in London</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>Medium - Dundurn mid-list title</t>
+          <t>Medium - LGBTQ+ literary debut</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -47281,14 +47285,14 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>Lives in St. Catharines, Ontario per Dundurn; confirm pub date | Review: no 2025–2027 publication date; Publication date not confirmed as 2025/2026</t>
+          <t>Confirm residence; listed on arsenalpulp.com/Events per assignment but snippet gave no location | Review: Residence/nationality not stated in results (novel set in London - may not be Canadian)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Dietrich Kalteis</t>
+          <t>Denise Da Costa</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -47296,16 +47300,20 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>And the Walls Came Down</t>
+        </is>
+      </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Crime fiction</t>
+          <t>Fiction (debut novel)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>publicity@ecwpress.com</t>
+          <t>publicity@dundurn.com</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -47315,33 +47323,33 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://ecwpress.com/pages/media-press</t>
+          <t>https://www.dundurn.com/contact</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
-          <t>ECW Press</t>
+          <t>Dundurn Press</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>https://ecwpress.com/collections/spring-2026</t>
+          <t>https://www.dundurn.com/blog_/t43181/p159409-essential-toronto-reading-list</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Listed among ECW Spring 2026 authors; latest confirmed title is The Get (June 2023)</t>
+          <t>Dundurn title</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>ECW bio: he enjoys life with his family on Canada's West Coast.</t>
+          <t>Debut novel about a woman returning to her hometown</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>High - crime novelist with a steady ECW backlist</t>
+          <t>Medium - Dundurn mid-list title</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -47366,7 +47374,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>Get the 2026 title and date from the ECW spring-2026 collection page. | Review: no 2025–2027 publication date; no book title; Spring 2026 title not named in search results</t>
+          <t>Lives in St. Catharines, Ontario per Dundurn; confirm pub date | Review: no 2025–2027 publication date; Publication date not confirmed as 2025/2026</t>
         </is>
       </c>
     </row>

</xml_diff>